<commit_message>
docs: Update Manual Book dan Revisi Test Case
</commit_message>
<xml_diff>
--- a/docs/testing/TC_Alert_Stok_Distribusi.xlsx
+++ b/docs/testing/TC_Alert_Stok_Distribusi.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="960" yWindow="500" windowWidth="32640" windowHeight="20500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-AS-UI (Visual)" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,14 +17,14 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TC-AS-FN (Negatif)'!$A$6:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TC-AS-EC (Edge Case)'!$A$6:$H$6</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,32 +34,31 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="001B5E20"/>
+      <family val="2"/>
+      <color rgb="FF1B5E20"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="001B5E20"/>
+      <color rgb="FF1B5E20"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00212121"/>
+      <family val="2"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -69,50 +67,44 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B5E20"/>
-        <bgColor rgb="001B5E20"/>
+        <fgColor rgb="FF1B5E20"/>
+        <bgColor rgb="FF1B5E20"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
-        <bgColor rgb="00E8F5E9"/>
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E7D32"/>
-        <bgColor rgb="002E7D32"/>
+        <fgColor rgb="FF2E7D32"/>
+        <bgColor rgb="FF2E7D32"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E3F2FD"/>
-        <bgColor rgb="00E3F2FD"/>
+        <fgColor rgb="FFE3F2FD"/>
+        <bgColor rgb="FFE3F2FD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C62828"/>
-        <bgColor rgb="00C62828"/>
+        <fgColor rgb="FFC62828"/>
+        <bgColor rgb="FFC62828"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006A1E55"/>
-        <bgColor rgb="006A1E55"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFDE7"/>
-        <bgColor rgb="00FFFDE7"/>
+        <fgColor rgb="FF6A1E55"/>
+        <bgColor rgb="FF6A1E55"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,16 +117,25 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -160,15 +161,9 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -531,8 +526,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -552,7 +547,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>SIMHPSB Web</t>
+          <t>SIMHP Web</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -632,6 +627,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -674,7 +670,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="65" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-001</t>
@@ -707,18 +703,18 @@
           <t>Judul 'Alert Stok' tampil di kiri atas area konten; subtitle 'Notifikasi otomatis saat stok mendekati batas minimum' tampil di bawah judul</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Halaman Alert Stok dibuka, judul 'Alert Stok' muncul di kiri atas dan subtitle 'Notifikasi otomatis saat stok mendekati batas minimum' tampil tepat di bawahnya. Tidak ada perbedaan dengan yang diharapkan.</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Judul 'Alert Stok' tampil di kiri atas area konten; subtitle 'Notifikasi otomatis saat stok mendekati batas minimum' tampil di bawah judul</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="91" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-002</t>
@@ -750,18 +746,18 @@
           <t>Panel menampilkan dua kartu: Beras (ikon padi hijau) dan Gabah (ikon padi oranye); masing-masing menampilkan label komoditas, nilai batas minimum, kapasitas, progress bar, dan persentase kapasitas</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Panel 'Konfigurasi Batas Minimum' tampil dengan dua kartu — Beras (ikon padi hijau) dan Gabah (ikon padi oranye). Masing-masing kartu menampilkan batas minimum, kapasitas, progress bar merah, dan persentase sisa kapasitas.</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Panel menampilkan dua kartu: Beras (ikon padi hijau) dan Gabah (ikon padi oranye); masing-masing menampilkan label komoditas, nilai batas minimum, kapasitas, progress bar, dan persentase kapasitas</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-003</t>
@@ -793,18 +789,18 @@
           <t>Badge 'Kritis' berwarna merah/pink tampil di pojok kanan atas setiap kartu komoditas yang stoknya di bawah batas minimum</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Saat stok Beras (100 kg) dan Gabah (500 kg) keduanya berada di bawah batas minimum masing-masing, badge 'Kritis' berwarna merah/pink muncul di pojok kanan atas kartu Beras maupun Gabah.</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Badge 'Kritis' berwarna merah/pink tampil di pojok kanan atas setiap kartu komoditas yang stoknya di bawah batas minimum</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="104" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-004</t>
@@ -836,18 +832,18 @@
           <t>Panel menampilkan tiga baris: 'Alert Aktif' (background merah/pink), 'Dalam Penanganan' (background kuning/oranye), 'Sudah Ditangani' (background hijau); setiap baris menampilkan jumlah dengan angka di sisi kanan</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>Panel 'Ringkasan Status Alert' tampil di sisi kanan dengan tiga baris: 'Alert Aktif' berlatar merah (angka 2), 'Dalam Penanganan' berlatar oranye (angka 1), dan 'Sudah Ditangani' berlatar hijau (angka 7).</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Panel menampilkan tiga baris: 'Alert Aktif' (background merah/pink), 'Dalam Penanganan' (background kuning/oranye), 'Sudah Ditangani' (background hijau); setiap baris menampilkan jumlah dengan angka di sisi kanan</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-005</t>
@@ -879,18 +875,18 @@
           <t>Tombol '⚙ Ubah' berwarna hijau tampil di pojok kanan atas panel Konfigurasi Batas Minimum; tombol dapat diklik</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Tombol '⚙ Ubah' berwarna hijau ditemukan di pojok kanan atas panel Konfigurasi Batas Minimum. Tombol berhasil diklik dan merespons tanpa error.</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Tombol '⚙ Ubah' berwarna hijau tampil di pojok kanan atas panel Konfigurasi Batas Minimum; tombol dapat diklik</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-006</t>
@@ -922,18 +918,18 @@
           <t>Tabel menampilkan kolom: WAKTU, KOMODITAS, STOK SAAT ALERT, BATAS MINIMUM, STATUS, DITANGANI OLEH, AKSI; semua header tampil sejajar dan terbaca</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Tabel Riwayat Alert menampilkan tujuh kolom header: WAKTU, KOMODITAS, STOK SAAT ALERT, BATAS MINIMUM, STATUS, DITANGANI OLEH, dan AKSI — semua sejajar dan terbaca jelas.</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Tabel menampilkan kolom: WAKTU, KOMODITAS, STOK SAAT ALERT, BATAS MINIMUM, STATUS, DITANGANI OLEH, AKSI; semua header tampil sejajar dan terbaca</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-007</t>
@@ -965,18 +961,18 @@
           <t>Dropdown 'Semua Status' tampil di pojok kanan atas tabel riwayat; dropdown dapat diklik untuk memfilter data</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Dropdown 'Semua Status' ditemukan di pojok kanan atas tabel riwayat. Saat diklik, dropdown terbuka dan menampilkan pilihan status: Aktif, Dalam Penanganan, Sudah Ditangani.</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="60" customHeight="1">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Dropdown 'Semua Status' tampil di pojok kanan atas tabel riwayat; dropdown dapat diklik untuk memfilter data</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="65" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-008</t>
@@ -1008,18 +1004,18 @@
           <t>Gabah: badge oranye/kuning; Beras: badge biru; Jagung: badge oranye berbeda; badge berbeda untuk setiap komoditas agar mudah dibedakan</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Badge komoditas di tabel riwayat tampil dengan warna berbeda: Gabah berwarna oranye/kuning, Beras berwarna biru muda, Jagung berwarna oranye lebih gelap. Ketiga komoditas mudah dibedakan secara visual.</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Gabah: badge oranye/kuning; Beras: badge biru; Jagung: badge oranye berbeda; badge berbeda untuk setiap komoditas agar mudah dibedakan</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-009</t>
@@ -1051,18 +1047,18 @@
           <t>'Aktif': badge merah; 'Dalam Penanganan': badge oranye/kuning; 'Sudah Ditangani': badge hijau dengan centang</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Kolom STATUS menampilkan badge berwarna sesuai kondisi: 'Aktif' merah, 'Dalam Penanganan' oranye, dan 'Sudah Ditangani' hijau dengan ikon centang di depannya.</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>'Aktif': badge merah; 'Dalam Penanganan': badge oranye/kuning; 'Sudah Ditangani': badge hijau dengan centang</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="78" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>TC-AS-UI-010</t>
@@ -1094,12 +1090,661 @@
           <t>Baris status 'Aktif': tombol '✓ Tandai Ditangani' berwarna hijau; baris status 'Dalam Penanganan': tombol '⚑ Selesai' berwarna abu; baris 'Sudah Ditangani': hanya teks '✓ Selesai'</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Kolom AKSI tiap baris menampilkan tombol yang sesuai statusnya: baris 'Aktif' punya tombol '✓ Tandai Ditangani' hijau, baris 'Dalam Penanganan' punya tombol '⚑ Selesai' abu, dan baris 'Sudah Ditangani' hanya teks '✓ Selesai' tanpa tombol klik.</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Baris status 'Aktif': tombol '✓ Tandai Ditangani' berwarna hijau; baris status 'Dalam Penanganan': tombol 'Selesai' berwarna abu; baris 'Sudah Ditangani': hanya teks '✓ Selesai'</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="65" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-001</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Halaman Stok Gudang dapat dibuka dan judul tampil dengan benar</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>1. Login sebagai Admin
+2. Klik menu 'Stok Gudang' di sidebar kiri
+3. Perhatikan judul halaman dan subtitle</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Judul 'Stok Gudang' tampil di kiri atas area konten beserta subtitle penjelasan halaman di bawahnya; menu 'Stok Gudang' pada sidebar dalam kondisi aktif/terpilih</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Judul 'Stok Gudang' tampil di kiri atas area konten beserta subtitle penjelasan halaman di bawahnya; menu 'Stok Gudang' pada sidebar dalam kondisi aktif/terpilih</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="65" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-002</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Ringkasan kartu stok per komoditas tampil di bagian atas halaman Stok Gudang</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Amati kartu ringkasan di bagian atas, sebelum tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Kartu ringkasan stok tampil untuk setiap komoditas dengan warna berbeda, masing-masing menunjukkan jumlah stok saat ini dalam kg</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Kartu ringkasan stok tampil untuk setiap komoditas dengan warna berbeda, masing-masing menunjukkan jumlah stok saat ini dalam kg</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="104" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-003</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Toolbar pencarian dan filter tampil lengkap di atas tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Amati area di atas tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Search bar dengan placeholder 'Cari tujuan, komoditas...' tampil; dropdown filter 'Semua Jenis' dan 'Semua Komoditas' tampil; date picker menampilkan tanggal saat ini; tombol hijau '+ Catat Transaksi' tampil di pojok kanan atas</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Search bar dengan placeholder 'Cari tujuan, komoditas...' tampil; dropdown filter 'Semua Jenis' dan 'Semua Komoditas' tampil; date picker menampilkan tanggal saat ini; tombol hijau '+ Catat Transaksi' tampil di pojok kanan atas</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="104" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-004</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Tabel Riwayat Transaksi Stok menampilkan semua kolom yang diperlukan</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Amati tabel riwayat transaksi di bagian bawah halaman</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Tabel menampilkan kolom: NO, TANGGAL, JENIS, KOMODITAS, JUMLAH (KG), TUJUAN/SUMBER, CATATAN, SALDO SETELAH, STATUS, BUKTI, DICATAT OLEH, AKSI; semua header tampil sejajar dan terbaca</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Tabel menampilkan kolom: NO, TANGGAL, JENIS, KOMODITAS, JUMLAH (KG), TUJUAN/SUMBER, CATATAN, SALDO SETELAH, STATUS, BUKTI, DICATAT OLEH, AKSI; semua header tampil sejajar dan terbaca</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="78" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-005</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Badge 'Jenis' transaksi tampil dengan warna dan ikon arah berbeda untuk Masuk dan Keluar</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Amati kolom JENIS pada tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Riwayat mengandung transaksi Masuk dan Keluar</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi 'Masuk' tampil dengan badge hijau berikon panah ke bawah (↓ Masuk); transaksi 'Keluar' tampil dengan badge merah/pink berikon panah ke atas (↑ Keluar)</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi 'Masuk' tampil dengan badge hijau berikon panah ke bawah (↓ Masuk); transaksi 'Keluar' tampil dengan badge merah/pink berikon panah ke atas (↑ Keluar)</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="78" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-006</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Badge komoditas pada tabel riwayat transaksi tampil berbeda warna untuk setiap komoditas</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Amati kolom KOMODITAS pada tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Riwayat mengandung data Beras, Gabah, Jagung</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Beras: badge biru; Gabah: badge oranye/kuning; Jagung: badge oranye berbeda; setiap komoditas memiliki warna badge yang konsisten dan mudah dibedakan</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Beras: badge biru; Gabah: badge oranye/kuning; Jagung: badge oranye berbeda; setiap komoditas memiliki warna badge yang konsisten dan mudah dibedakan</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="91" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-007</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Badge status transaksi tampil sesuai kondisi Aktif dan Dibatalkan</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Amati kolom STATUS pada tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Riwayat mengandung transaksi berstatus Aktif dan Dibatalkan</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Status 'Aktif' tampil dengan badge hijau; status 'Dibatalkan' tampil dengan badge abu-abu, dan seluruh data pada baris tersebut (tanggal, jumlah, saldo setelah) tampil dengan format teks tercoret (strikethrough)</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Status 'Aktif' tampil dengan badge hijau; status 'Dibatalkan' tampil dengan badge abu-abu, dan seluruh data pada baris tersebut (tanggal, jumlah, saldo setelah) tampil dengan format teks tercoret (strikethrough)</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="65" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-008</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Kolom BUKTI menampilkan thumbnail foto jika tersedia atau tanda '-' bila tidak ada</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Amati kolom BUKTI pada tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Terdapat transaksi dengan dan tanpa foto bukti pengiriman</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Baris dengan foto bukti menampilkan thumbnail/ikon gambar yang dapat diklik; baris tanpa foto bukti menampilkan tanda '-'</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Baris dengan foto bukti menampilkan thumbnail/ikon gambar yang dapat diklik; baris tanpa foto bukti menampilkan tanda '-'</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="91" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-009</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Tombol aksi pada kolom AKSI tampil sesuai status transaksi</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Amati kolom AKSI untuk baris berstatus Aktif dan Dibatalkan</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Terdapat transaksi berstatus Aktif dan Dibatalkan</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Baris status 'Aktif' menampilkan ikon mata (lihat) dan ikon silang merah/pink (hapus); baris status 'Dibatalkan' menampilkan ikon mata (lihat) dan ikon pemulihan hijau (restore) sebagai pengganti ikon hapus</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Baris status 'Aktif' menampilkan ikon mata (lihat) dan ikon silang merah/pink (hapus); baris status 'Dibatalkan' menampilkan ikon mata (lihat) dan ikon pemulihan hijau (restore) sebagai pengganti ikon hapus</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="143" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-010</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Modal 'Catat Transaksi Stok' menampilkan seluruh field input yang diperlukan</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Klik tombol '+ Catat Transaksi'
+3. Amati field-field pada modal yang terbuka</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Modal 'Catat Transaksi Stok' menampilkan field: Jenis Transaksi*, Komoditas*, Jumlah (kg)*, Tanggal, Tujuan Distribusi*, Sumber/Keterangan*, Catatan Tambahan (opsional), serta unggah Foto Bukti Pengiriman (jpg, png, webp – maks 2MB); tombol 'Batal' dan 'Simpan' tampil di bagian bawah modal</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Modal 'Catat Transaksi Stok' menampilkan field: Jenis Transaksi*, Komoditas*, Jumlah (kg)*, Tanggal, Tujuan Distribusi*, Sumber/Keterangan*, Catatan Tambahan (opsional), serta unggah Foto Bukti Pengiriman (jpg, png, webp – maks 2MB); tombol 'Batal' dan 'Simpan' tampil di bagian bawah modal</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="117" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-011</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Halaman 'Detail Transaksi Stok' menampilkan seluruh informasi transaksi secara lengkap</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Klik ikon mata (lihat) pada salah satu baris transaksi
+3. Amati halaman detail yang terbuka</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Halaman 'Detail Transaksi Stok' menampilkan tautan '← Kembali ke Stok Gudang', serta informasi Tanggal Transaksi, Jenis Transaksi, Komoditas, Jumlah, Saldo Setelah, Tujuan/Sumber, Catatan, Foto Bukti, Dicatat Oleh, ID Transaksi, Dibuat, dan Terakhir Diperbarui</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Halaman 'Detail Transaksi Stok' menampilkan tautan '← Kembali ke Stok Gudang', serta informasi Tanggal Transaksi, Jenis Transaksi, Komoditas, Jumlah, Saldo Setelah, Tujuan/Sumber, Catatan, Foto Bukti, Dicatat Oleh, ID Transaksi, Dibuat, dan Terakhir Diperbarui</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="91" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-UI-012</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – UI</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Foto Bukti pada halaman detail dapat dilihat dalam ukuran penuh tanpa meninggalkan halaman</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman 'Detail Transaksi Stok' pada transaksi yang memiliki foto bukti
+2. Klik thumbnail Foto Bukti</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Gambar tampil dalam ukuran penuh melalui lightbox/modal pada halaman yang sama, tanpa membuka tab atau halaman baru, sesuai keterangan 'Klik gambar untuk melihat ukuran penuh tanpa meninggalkan halaman.'</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Gambar tampil dalam ukuran penuh melalui lightbox/modal pada halaman yang sama, tanpa membuka tab atau halaman baru, sesuai keterangan 'Klik gambar untuk melihat ukuran penuh tanpa meninggalkan halaman.'</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="78" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-UI-001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – UI</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Halaman 'Manajemen Tujuan Distribusi' dapat dibuka dan judul tampil dengan benar</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>1. Login sebagai Admin
+2. Klik menu 'Tujuan Distribusi' di sidebar kiri
+3. Perhatikan judul halaman dan subtitle</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Judul 'Manajemen Tujuan Distribusi' tampil di kiri atas area konten; subtitle 'Tambah/hapus tujuan distribusi yang digunakan pada pencatatan stok' tampil di bawah judul</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Judul 'Manajemen Tujuan Distribusi' tampil di kiri atas area konten; subtitle 'Tambah/hapus tujuan distribusi yang digunakan pada pencatatan stok' tampil di bawah judul</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="117" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-UI-002</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – UI</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Tabel 'Daftar Tujuan Distribusi' tampil dengan kolom yang lengkap</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Manajemen Tujuan Distribusi
+2. Amati tabel daftar tujuan</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Panel 'Daftar Tujuan Distribusi' dengan subtitle 'Semua tujuan yang tersedia untuk transaksi keluar' tampil; tabel menampilkan kolom #, NAMA TUJUAN, DIBUAT, AKSI; setiap baris memiliki tombol 'Hapus' berwarna merah/pink dengan ikon tempat sampah</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Panel 'Daftar Tujuan Distribusi' dengan subtitle 'Semua tujuan yang tersedia untuk transaksi keluar' tampil; tabel menampilkan kolom #, NAMA TUJUAN, DIBUAT, AKSI; setiap baris memiliki tombol 'Hapus' berwarna merah/pink dengan ikon tempat sampah</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="78" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-UI-003</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – UI</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Tombol '+ Tambah Tujuan' tersedia dan dapat diklik</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Manajemen Tujuan Distribusi
+2. Cari tombol '+ Tambah Tujuan' di pojok kanan atas</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Tombol '+ Tambah Tujuan' berwarna hijau tampil di pojok kanan atas panel Daftar Tujuan Distribusi; tombol dapat diklik untuk membuka form tambah tujuan baru</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Tombol '+ Tambah Tujuan' berwarna hijau tampil di pojok kanan atas panel Daftar Tujuan Distribusi; tombol dapat diklik untuk membuka form tambah tujuan baru</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1117,8 +1762,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H39"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -1138,7 +1783,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>SIMHPSB Web</t>
+          <t>SIMHP Web</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1174,7 +1819,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Description</t>
@@ -1187,7 +1832,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Test Case Version</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1196,7 +1841,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="56" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Test Objective</t>
@@ -1218,6 +1863,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -1260,7 +1906,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="91" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-001</t>
@@ -1296,18 +1942,18 @@
           <t>Status baris berubah menjadi 'Sudah Ditangani'; kolom 'Ditangani Oleh' terisi dengan nama Admin yang login; tombol aksi berubah menjadi '✓ Selesai'; jumlah 'Alert Aktif' di Ringkasan Status berkurang</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Setelah klik '✓ Tandai Ditangani' pada alert Gabah yang aktif, status baris langsung berubah jadi 'Sudah Ditangani'. Kolom 'Ditangani Oleh' terisi 'Admin SIMHPSB' dan jumlah Alert Aktif di panel Ringkasan turun dari 2 jadi 1.</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Status baris berubah menjadi 'Sudah Ditangani'; kolom 'Ditangani Oleh' terisi dengan nama Admin yang login; tombol aksi berubah menjadi '✓ Selesai'; jumlah 'Alert Aktif' di Ringkasan Status berkurang</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-002</t>
@@ -1342,18 +1988,18 @@
           <t>Status berubah menjadi 'Sudah Ditangani'; nama admin dicatat di kolom Ditangani Oleh; counter Ringkasan berkurang di Alert Aktif dan bertambah di Sudah Ditangani</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Alert Beras (stok -1.108.900 kg) berhasil ditandai ditangani. Status berubah ke 'Sudah Ditangani', nama Admin SIMHPSB tercatat di kolom Ditangani Oleh, dan Ringkasan diperbarui: Alert Aktif berkurang, Sudah Ditangani bertambah.</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Status berubah menjadi 'Sudah Ditangani'; nama admin dicatat di kolom Ditangani Oleh; counter Ringkasan berkurang di Alert Aktif dan bertambah di Sudah Ditangani</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="65" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-003</t>
@@ -1388,18 +2034,18 @@
           <t>Status berubah menjadi 'Sudah Ditangani'; jumlah 'Dalam Penanganan' di Ringkasan berkurang 1; jumlah 'Sudah Ditangani' bertambah 1</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Klik '⚑ Selesai' pada alert Jagung yang berstatus 'Dalam Penanganan' mengubah statusnya jadi 'Sudah Ditangani'. Counter 'Dalam Penanganan' di Ringkasan berkurang 1 dan 'Sudah Ditangani' bertambah 1.</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Status berubah menjadi 'Sudah Ditangani'; jumlah 'Dalam Penanganan' di Ringkasan berkurang 1; jumlah 'Sudah Ditangani' bertambah 1</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="65" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-004</t>
@@ -1433,18 +2079,18 @@
           <t>Tabel hanya menampilkan baris dengan status 'Aktif'; baris dengan status lain (Dalam Penanganan, Sudah Ditangani) tidak muncul</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>Setelah memilih filter 'Aktif' dari dropdown, tabel hanya menampilkan baris-baris berstatus Aktif. Baris dengan status Dalam Penanganan dan Sudah Ditangani tidak muncul sama sekali.</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Tabel hanya menampilkan baris dengan status 'Aktif'; baris dengan status lain (Dalam Penanganan, Sudah Ditangani) tidak muncul</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-005</t>
@@ -1477,18 +2123,18 @@
           <t>Tabel hanya menampilkan baris berstatus 'Dalam Penanganan'; baris Aktif dan Sudah Ditangani tersembunyi</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Filter 'Dalam Penanganan' dipilih, tabel langsung menampilkan 1 baris dengan status Dalam Penanganan saja. Semua baris berstatus Aktif dan Sudah Ditangani menghilang dari tampilan.</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Tabel hanya menampilkan baris berstatus 'Dalam Penanganan'; baris Aktif dan Sudah Ditangani tersembunyi</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-006</t>
@@ -1521,18 +2167,18 @@
           <t>Tabel hanya menampilkan data berstatus 'Sudah Ditangani'; kolom Ditangani Oleh terisi nama petugas</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Filter 'Sudah Ditangani' aktif, tabel menampilkan baris-baris yang sudah selesai ditangani. Kolom 'Ditangani Oleh' tiap baris sudah terisi nama Admin SIMHPSB atau Petugas SIMHPSB.</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Tabel hanya menampilkan data berstatus 'Sudah Ditangani'; kolom Ditangani Oleh terisi nama petugas</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="65" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-007</t>
@@ -1566,18 +2212,18 @@
           <t>Nilai batas minimum Beras berubah menjadi 600 kg di panel konfigurasi; sistem menggunakan nilai baru sebagai acuan pemicu alert</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Batas minimum Beras berhasil diubah menjadi 600 kg. Setelah disimpan, kartu Beras di panel Konfigurasi langsung menampilkan angka 600 kg sebagai batas minimum yang baru.</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="60" customHeight="1">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Nilai batas minimum Beras berubah menjadi 600 kg di panel konfigurasi; sistem menggunakan nilai baru sebagai acuan pemicu alert</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-008</t>
@@ -1611,18 +2257,18 @@
           <t>Nilai batas minimum Gabah berubah menjadi 1.500 kg; panel konfigurasi menampilkan nilai terbaru</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Batas minimum Gabah berhasil diperbarui menjadi 1.500 kg. Panel Konfigurasi Batas Minimum menampilkan nilai 1.500 kg setelah simpan, menggantikan nilai sebelumnya.</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Nilai batas minimum Gabah berubah menjadi 1.500 kg; panel konfigurasi menampilkan nilai terbaru</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="65" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-009</t>
@@ -1654,18 +2300,18 @@
           <t>Jumlah di Ringkasan Status Alert (Alert Aktif, Dalam Penanganan, Sudah Ditangani) sesuai dengan jumlah baris di tabel; tidak ada selisih</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Jumlah di panel Ringkasan dicocokkan manual dengan baris di tabel: Alert Aktif = 2 baris, Dalam Penanganan = 1 baris, Sudah Ditangani = 7 baris. Ketiganya sesuai, tidak ada selisih.</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Jumlah di Ringkasan Status Alert (Alert Aktif, Dalam Penanganan, Sudah Ditangani) sesuai dengan jumlah baris di tabel; tidak ada selisih</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="65" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-010</t>
@@ -1698,18 +2344,18 @@
           <t>Progress bar Beras menampilkan ±1% terisi; progress bar Gabah menampilkan ±10% terisi; angka persentase di bawah progress bar sesuai perhitungan</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Progress bar Beras terisi sekitar 1% (100 kg dari kapasitas 10.000 kg) dan Gabah sekitar 10% (500 kg dari 5.000 kg). Angka persentase di bawah masing-masing bar sesuai dengan hasil hitungan manual.</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1">
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Progress bar Beras menampilkan ±1% terisi; progress bar Gabah menampilkan ±10% terisi; angka persentase di bawah progress bar sesuai perhitungan</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-011</t>
@@ -1741,18 +2387,18 @@
           <t>Baris paling atas memiliki tanggal/waktu paling baru; baris paling bawah memiliki tanggal/waktu paling lama</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Urutan waktu di tabel riwayat terurut dari terbaru ke terlama. Baris pertama bertanggal '27 May 2026 08:00' dan baris terakhir '25 May 2026 10:07' — urutan descending sudah benar.</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Baris paling atas memiliki tanggal/waktu paling baru; baris paling bawah memiliki tanggal/waktu paling lama</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FP-012</t>
@@ -1784,12 +2430,948 @@
           <t>Nilai stok negatif ditampilkan dengan warna merah; nilai stok normal (positif) ditampilkan dengan warna hitam/abu biasa</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>Nilai negatif seperti -1.108.900 kg dan -1.000 kg di kolom STOK SAAT ALERT ditampilkan berwarna merah. Nilai positif seperti 500 kg tampil dengan warna teks normal/hitam.</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Nilai stok negatif ditampilkan dengan warna merah; nilai stok normal (positif) ditampilkan dengan warna hitam/abu biasa</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="91" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-001</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Mencatat transaksi 'Keluar' baru berhasil tersimpan dan saldo berkurang sesuai jumlah</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>1. Login sebagai Admin
+2. Buka halaman Stok Gudang
+3. Klik '+ Catat Transaksi'
+4. Pilih Jenis Transaksi 'Keluar', isi Komoditas, Jumlah, Tujuan Distribusi, dan Sumber/Keterangan
+5. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Jenis: Keluar | Komoditas: Beras | Jumlah: 200 kg | Tujuan Distribusi: MBG Dapur 1</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi baru muncul di baris teratas tabel riwayat dengan status 'Aktif'; Saldo Setelah berkurang 200 kg dari saldo sebelumnya; data Jenis, Komoditas, Jumlah, dan Tujuan sesuai input</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi baru muncul di baris teratas tabel riwayat dengan status 'Aktif'; Saldo Setelah berkurang 200 kg dari saldo sebelumnya; data Jenis, Komoditas, Jumlah, dan Tujuan sesuai input</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="91" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-002</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Mencatat transaksi 'Masuk' baru berhasil tersimpan dan saldo bertambah sesuai jumlah</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Klik '+ Catat Transaksi'
+3. Pilih Jenis Transaksi 'Masuk', isi Komoditas, Jumlah, dan Sumber/Keterangan
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Jenis: Masuk | Komoditas: Gabah | Jumlah: 500 kg | Sumber: Petani Budi</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi baru muncul di baris teratas tabel riwayat dengan status 'Aktif'; Saldo Setelah bertambah 500 kg dari saldo sebelumnya; kolom Tujuan/Sumber menampilkan 'Petani Budi'</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi baru muncul di baris teratas tabel riwayat dengan status 'Aktif'; Saldo Setelah bertambah 500 kg dari saldo sebelumnya; kolom Tujuan/Sumber menampilkan 'Petani Budi'</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="78" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-003</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Field Tanggal pada form Catat Transaksi otomatis menggunakan waktu saat tombol Simpan diklik bila tidak diubah</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Biarkan field Tanggal tanpa diubah
+3. Lengkapi field wajib lainnya
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Tanggal: tidak diubah (default)</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi tersimpan dengan Tanggal Transaksi sesuai waktu nyata saat tombol Simpan diklik, sesuai keterangan 'Waktu akan terisi otomatis saat menyimpan jika Anda tidak mengubahnya.'</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi tersimpan dengan Tanggal Transaksi sesuai waktu nyata saat tombol Simpan diklik, sesuai keterangan 'Waktu akan terisi otomatis saat menyimpan jika Anda tidak mengubahnya.'</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="65" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-004</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Mengubah field Tanggal secara manual pada form Catat Transaksi tersimpan sesuai input pengguna</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Ubah field Tanggal ke tanggal/waktu tertentu
+3. Lengkapi field wajib lainnya
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Tanggal diubah ke: 10/06/2026, 09:00</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi tersimpan dengan Tanggal Transaksi sesuai nilai yang diinput pengguna (10/06/2026 09:00), bukan waktu sistem saat ini</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi tersimpan dengan Tanggal Transaksi sesuai nilai yang diinput pengguna (10/06/2026 09:00), bukan waktu sistem saat ini</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="78" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-005</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Mengunggah Foto Bukti Pengiriman yang valid berhasil tersimpan dan tampil di tabel serta halaman detail</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Lengkapi field wajib
+3. Klik 'Pilih File' pada Foto Bukti Pengiriman dan pilih file gambar
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>File: bukti.jpg (500 KB, format jpg)</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi tersimpan; kolom BUKTI pada tabel riwayat menampilkan thumbnail gambar; halaman Detail Transaksi Stok menampilkan Foto Bukti yang sama</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi tersimpan; kolom BUKTI pada tabel riwayat menampilkan thumbnail gambar; halaman Detail Transaksi Stok menampilkan Foto Bukti yang sama</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="104" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-006</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Klik ikon mata (lihat) pada baris transaksi menampilkan halaman Detail Transaksi Stok dengan data yang sesuai</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Klik ikon mata pada salah satu baris transaksi</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Halaman Detail Transaksi Stok terbuka menampilkan data (Tanggal, Jenis, Komoditas, Jumlah, Saldo Setelah, Tujuan/Sumber, Catatan, Dicatat Oleh, ID Transaksi, Dibuat, Terakhir Diperbarui) yang sesuai dengan baris yang dipilih</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Halaman Detail Transaksi Stok terbuka menampilkan data (Tanggal, Jenis, Komoditas, Jumlah, Saldo Setelah, Tujuan/Sumber, Catatan, Dicatat Oleh, ID Transaksi, Dibuat, Terakhir Diperbarui) yang sesuai dengan baris yang dipilih</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="117" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-007</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Klik ikon hapus (X) pada transaksi Aktif membatalkan transaksi tanpa menghapus data secara permanen</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Klik ikon silang (Hapus) pada baris transaksi berstatus 'Aktif'
+3. Konfirmasi jika ada dialog konfirmasi
+4. Amati perubahan pada baris tersebut</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi: Beras | Keluar | 200 kg | Status awal: Aktif</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Status baris berubah menjadi 'Dibatalkan'; data pada baris (tanggal, jumlah, saldo setelah) tampil tercoret; ikon Hapus berubah menjadi ikon pemulihan (restore) hijau; saldo stok komoditas terkait dihitung ulang seolah transaksi tersebut tidak terjadi</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Status baris berubah menjadi 'Dibatalkan'; data pada baris (tanggal, jumlah, saldo setelah) tampil tercoret; ikon Hapus berubah menjadi ikon pemulihan (restore) hijau; saldo stok komoditas terkait dihitung ulang seolah transaksi tersebut tidak terjadi</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="104" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-008</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Klik ikon pemulihan (restore) pada transaksi Dibatalkan mengembalikan status menjadi Aktif</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Temukan baris transaksi berstatus 'Dibatalkan'
+3. Klik ikon pemulihan (restore) berwarna hijau
+4. Amati perubahan pada baris tersebut</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi: status awal Dibatalkan</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Status baris berubah kembali menjadi 'Aktif'; format teks tercoret hilang; ikon restore berubah kembali menjadi ikon Hapus; saldo stok komoditas terkait dihitung ulang dengan memperhitungkan kembali transaksi tersebut</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Status baris berubah kembali menjadi 'Aktif'; format teks tercoret hilang; ikon restore berubah kembali menjadi ikon Hapus; saldo stok komoditas terkait dihitung ulang dengan memperhitungkan kembali transaksi tersebut</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="78" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-009</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Setelah pada transaksi-transaksi sesudahnya otomatis dihitung ulang ketika transaksi sebelumnya dibatalkan/dipulihkan</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>1. Catat beberapa transaksi berurutan untuk komoditas yang sama
+2. Batalkan salah satu transaksi di tengah urutan waktu
+3. Periksa kolom Saldo Setelah pada transaksi-transaksi sesudahnya</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Minimal 3 transaksi berurutan untuk komoditas yang sama</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Setelah pada seluruh transaksi yang tercatat setelah transaksi yang dibatalkan otomatis menyesuaikan, sehingga tetap konsisten dengan urutan transaksi yang masih Aktif</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Saldo Setelah pada seluruh transaksi yang tercatat setelah transaksi yang dibatalkan otomatis menyesuaikan, sehingga tetap konsisten dengan urutan transaksi yang masih Aktif</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="78" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-010</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Filter 'Semua Jenis' dan 'Semua Komoditas' dapat memfilter tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Pilih jenis tertentu pada dropdown 'Semua Jenis' (mis. Keluar)
+3. Pilih komoditas tertentu pada dropdown 'Semua Komoditas' (mis. Beras)
+4. Amati data yang ditampilkan</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Filter Jenis: Keluar | Filter Komoditas: Beras</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Tabel hanya menampilkan baris transaksi dengan Jenis 'Keluar' dan Komoditas 'Beras'; baris lain yang tidak sesuai filter tersembunyi</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Tabel hanya menampilkan baris transaksi dengan Jenis 'Keluar' dan Komoditas 'Beras'; baris lain yang tidak sesuai filter tersembunyi</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="65" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-011</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Pencarian pada search bar menampilkan hasil sesuai kata kunci tujuan atau komoditas</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Ketik kata kunci pada search bar 'Cari tujuan, komoditas...'
+3. Amati hasil yang ditampilkan</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Kata kunci: 'MBG Dapur 1'</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Tabel hanya menampilkan baris transaksi yang kolom Tujuan/Sumber atau Komoditasnya cocok dengan kata kunci 'MBG Dapur 1'</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Tabel hanya menampilkan baris transaksi yang kolom Tujuan/Sumber atau Komoditasnya cocok dengan kata kunci 'MBG Dapur 1'</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="52" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-FP-001</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – Fungsional</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Menambahkan Tujuan Distribusi baru berhasil tersimpan dan muncul di daftar</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Manajemen Tujuan Distribusi
+2. Klik '+ Tambah Tujuan'
+3. Isi nama tujuan baru
+4. Simpan</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Nama Tujuan: 'Toko Sumber Rejeki'</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan baru 'Toko Sumber Rejeki' muncul di tabel Daftar Tujuan Distribusi dengan tanggal Dibuat hari ini</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Tujuan baru 'Toko Sumber Rejeki' muncul di tabel Daftar Tujuan Distribusi dengan tanggal Dibuat hari ini</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="65" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-FP-002</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – Fungsional</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi yang baru ditambahkan langsung tersedia pada dropdown 'Tujuan Distribusi' di form Catat Transaksi</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>1. Tambahkan tujuan baru melalui Manajemen Tujuan Distribusi
+2. Buka halaman Stok Gudang
+3. Klik '+ Catat Transaksi'
+4. Buka dropdown 'Tujuan Distribusi'</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan baru: 'Toko Sumber Rejeki'</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Dropdown 'Tujuan Distribusi' pada form Catat Transaksi menampilkan opsi 'Toko Sumber Rejeki' sebagai pilihan baru</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Dropdown 'Tujuan Distribusi' pada form Catat Transaksi menampilkan opsi 'Toko Sumber Rejeki' sebagai pilihan baru</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="65" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-FP-003</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – Fungsional</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Menghapus Tujuan Distribusi yang ada berhasil dan tujuan tersebut tidak lagi muncul di daftar maupun dropdown</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Manajemen Tujuan Distribusi
+2. Klik tombol 'Hapus' pada salah satu tujuan
+3. Konfirmasi jika ada dialog konfirmasi
+4. Periksa tabel daftar tujuan dan dropdown Tujuan Distribusi pada form Catat Transaksi</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan yang dihapus: 'Toko Rudi'</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan 'Toko Rudi' tidak lagi tampil di tabel Daftar Tujuan Distribusi maupun pada dropdown 'Tujuan Distribusi' di form Catat Transaksi</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Tujuan 'Toko Rudi' tidak lagi tampil di tabel Daftar Tujuan Distribusi maupun pada dropdown 'Tujuan Distribusi' di form Catat Transaksi</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="52" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-012</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Pengguna dapat menutup halaman Detail Transaksi Stok dan kembali ke halaman Stok Gudang</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Klik ikon mata pada salah satu baris transaksi
+3. Pada halaman Detail Transaksi Stok, klik tautan '← Kembali ke Stok Gudang'</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Pengguna diarahkan kembali ke halaman Stok Gudang; tabel riwayat transaksi tampil seperti semula tanpa perubahan data</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Pengguna diarahkan kembali ke halaman Stok Gudang; tabel riwayat transaksi tampil seperti semula tanpa perubahan data</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="78" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-013</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Detail transaksi yang ditampilkan sesuai dengan baris data yang dipilih (tidak tertukar antar transaksi)</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik ikon mata pada Transaksi A, catat data yang tampil
+2. Kembali ke Stok Gudang
+3. Klik ikon mata pada Transaksi B yang berbeda
+4. Bandingkan data kedua halaman detail</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi A: Beras, Keluar, 200 kg; Transaksi B: Gabah, Masuk, 500 kg</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Data pada masing-masing halaman detail (Tanggal, Jenis, Komoditas, Jumlah, Saldo Setelah, dll.) sesuai dengan transaksi yang dipilih; tidak ada data yang tertukar</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Data pada masing-masing halaman detail (Tanggal, Jenis, Komoditas, Jumlah, Saldo Setelah, dll.) sesuai dengan transaksi yang dipilih; tidak ada data yang tertukar</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="52" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-014</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Foto form transaksi 'Keluar' yang tersedia ditampilkan pada halaman Detail Transaksi Stok</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik ikon mata pada transaksi berjenis 'Keluar' yang memiliki foto form terlampir
+2. Amati bagian Foto Bukti pada halaman detail</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi: Keluar, Beras, 200 kg, dengan foto form terlampir</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Foto form transaksi ditampilkan sebagai thumbnail pada bagian 'Foto Bukti' di halaman Detail Transaksi Stok</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Foto form transaksi ditampilkan sebagai thumbnail pada bagian 'Foto Bukti' di halaman Detail Transaksi Stok</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="52" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-015</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Foto form transaksi pada halaman detail dapat diperbesar agar isi form terlihat jelas</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Detail Transaksi Stok pada transaksi 'Keluar' yang memiliki foto form
+2. Klik thumbnail Foto Bukti</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Foto form tampil dalam ukuran penuh (lightbox) tanpa meninggalkan halaman, sehingga isi form dapat dibaca dengan jelas</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Foto form tampil dalam ukuran penuh (lightbox) tanpa meninggalkan halaman, sehingga isi form dapat dibaca dengan jelas</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="104" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-016</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Klik ikon silang (Hapus) pada transaksi Masuk berstatus Aktif membatalkan transaksi tanpa menghapus data secara permanen</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Stok Gudang
+2. Klik ikon silang (Hapus) pada baris transaksi 'Masuk' berstatus 'Aktif'
+3. Konfirmasi jika ada dialog konfirmasi
+4. Amati perubahan pada baris tersebut</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi: Gabah | Masuk | 500 kg | Status awal: Aktif</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Status baris berubah menjadi 'Dibatalkan'; data pada baris tampil tercoret; ikon Hapus berubah menjadi ikon pemulihan (restore) hijau; saldo stok komoditas terkait dihitung ulang seolah transaksi tersebut tidak terjadi</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Status baris berubah menjadi 'Dibatalkan'; data pada baris tampil tercoret; ikon Hapus berubah menjadi ikon pemulihan (restore) hijau; saldo stok komoditas terkait dihitung ulang seolah transaksi tersebut tidak terjadi</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="78" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-017</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Status Dibatalkan pada transaksi tetap konsisten setelah halaman Stok Gudang di-refresh/reload</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>1. Batalkan salah satu transaksi hingga berstatus 'Dibatalkan'
+2. Refresh/reload halaman Stok Gudang
+3. Amati status transaksi tersebut pada tabel riwayat</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi yang dibatalkan: Beras, Keluar, 200 kg</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Setelah reload, transaksi tersebut tetap tampil pada tabel dengan status 'Dibatalkan' dan format tercoret; tidak kembali ke status 'Aktif' maupun hilang dari tabel</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Setelah reload, transaksi tersebut tetap tampil pada tabel dengan status 'Dibatalkan' dan format tercoret; tidak kembali ke status 'Aktif' maupun hilang dari tabel</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="78" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FP-018</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Fungsional</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Membatalkan beberapa transaksi sekaligus (lebih dari satu baris) berfungsi dengan benar</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik ikon Hapus pada baris ke-1
+2. Klik ikon Hapus pada baris ke-3
+3. Klik ikon Hapus pada baris ke-5
+4. Amati tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>3 baris dibatalkan sekaligus (baris ke-1, ke-3, ke-5)</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Ketiga baris yang diklik berubah status menjadi 'Dibatalkan' dengan format tercoret; baris lain tetap berstatus 'Aktif' seperti semula; tidak ada error atau data yang hilang</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Ketiga baris yang diklik berubah status menjadi 'Dibatalkan' dengan format tercoret; baris lain tetap berstatus 'Aktif' seperti semula; tidak ada error atau data yang hilang</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1807,8 +3389,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -1828,7 +3410,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>SIMHPSB Web</t>
+          <t>SIMHP Web</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1864,7 +3446,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Description</t>
@@ -1886,7 +3468,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="56" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Test Objective</t>
@@ -1908,6 +3490,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
@@ -1950,7 +3533,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="65" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-001</t>
@@ -1983,18 +3566,18 @@
           <t>Tidak ada tombol aktif untuk menandai ulang; hanya teks '✓ Selesai' yang ditampilkan; tidak ada aksi yang dapat dilakukan pada alert yang sudah selesai</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Dicek baris dengan status 'Sudah Ditangani' — kolom AKSI hanya menampilkan teks '✓ Selesai' tanpa tombol yang bisa diklik. Tidak ada opsi untuk menandai ulang alert yang sudah selesai.</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Tidak ada tombol aktif untuk menandai ulang; hanya teks '✓ Selesai' yang ditampilkan; tidak ada aksi yang dapat dilakukan pada alert yang sudah selesai</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-002</t>
@@ -2027,18 +3610,18 @@
           <t>Sistem menampilkan pesan validasi error bahwa batas minimum tidak boleh 0 atau negatif; data tidak tersimpan</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Nilai 0 dimasukkan sebagai batas minimum Beras lalu klik Simpan. Sistem menampilkan pesan validasi bahwa nilai tidak boleh 0 atau negatif. Batas minimum Beras tidak berubah.</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error bahwa batas minimum tidak boleh 0 atau negatif; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="39" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-003</t>
@@ -2071,18 +3654,18 @@
           <t>Sistem menampilkan validasi error; nilai negatif tidak diterima untuk batas minimum stok</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Nilai -500 dimasukkan sebagai batas minimum Gabah lalu klik Simpan. Sistem langsung memunculkan pesan validasi error. Nilai negatif ditolak dan batas minimum Gabah tetap pada nilai semula.</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan validasi error; nilai negatif tidak diterima untuk batas minimum stok</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="39" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-004</t>
@@ -2115,18 +3698,18 @@
           <t>Field menolak input non-numerik; sistem menampilkan error validasi; data tidak tersimpan</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>Teks 'abc' diketik pada field batas minimum — field bertipe number langsung menolak input huruf. Klik Simpan tetap tidak memproses data dan muncul pesan validasi.</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Field menolak input non-numerik; sistem menampilkan error validasi; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-005</t>
@@ -2159,18 +3742,18 @@
           <t>Sistem menampilkan error atau warning bahwa batas minimum tidak boleh melebihi kapasitas gudang; data tidak tersimpan</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Nilai 15.000 diinput sebagai batas minimum Beras (kapasitas 10.000 kg). Sistem menampilkan peringatan bahwa batas minimum tidak boleh melebihi kapasitas gudang. Data tidak tersimpan.</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan error atau warning bahwa batas minimum tidak boleh melebihi kapasitas gudang; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="65" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-006</t>
@@ -2202,18 +3785,18 @@
           <t>Tabel menampilkan pesan informatif seperti 'Tidak ada data untuk status ini' atau tabel kosong dengan pesan; tidak ada error atau crash</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Filter 'Dalam Penanganan' dipilih saat tidak ada data dengan status tersebut. Tabel menampilkan area kosong dengan pesan bahwa tidak ada data untuk status ini. Tidak ada crash maupun error.</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Tabel menampilkan pesan informatif seperti 'Tidak ada data untuk status ini' atau tabel kosong dengan pesan; tidak ada error atau crash</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="65" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-007</t>
@@ -2246,18 +3829,18 @@
           <t>Tombol 'Ubah' tidak tampil ATAU jika diklik muncul pesan 'Akses ditolak'; Petugas tidak dapat mengubah konfigurasi batas minimum</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Login sebagai Petugas lalu buka Alert Stok — tombol '⚙ Ubah' tidak tampil di panel Konfigurasi Batas Minimum. Petugas tidak bisa mengubah konfigurasi apapun di halaman ini.</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="60" customHeight="1">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Tombol 'Ubah' tidak tampil ATAU jika diklik muncul pesan 'Akses ditolak'; Petugas tidak dapat mengubah konfigurasi batas minimum</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="65" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-008</t>
@@ -2289,18 +3872,18 @@
           <t>Nilai ditampilkan utuh dengan pemisah ribuan yang benar; tidak ada truncation atau error tampilan; angka tetap terbaca di tabel</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Nilai -1.108.900 kg tampil utuh di kolom STOK SAAT ALERT dengan pemisah ribuan yang benar. Tidak ada pemotongan angka maupun error tampilan meski nilainya sangat besar.</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Nilai ditampilkan utuh dengan pemisah ribuan yang benar; tidak ada truncation atau error tampilan; angka tetap terbaca di tabel</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="65" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>TC-AS-FN-009</t>
@@ -2333,12 +3916,595 @@
           <t>Status hanya berubah satu kali menjadi 'Sudah Ditangani'; tidak ada duplikasi entri atau error; counter Ringkasan hanya berkurang 1</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Tombol '✓ Tandai Ditangani' diklik dua kali berturut-turut dengan cepat. Status tetap berubah hanya satu kali menjadi 'Sudah Ditangani'. Counter Ringkasan hanya berkurang 1, tidak ada duplikasi.</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Status hanya berubah satu kali menjadi 'Sudah Ditangani'; tidak ada duplikasi entri atau error; counter Ringkasan hanya berkurang 1</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-001</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Menyimpan transaksi tanpa memilih Jenis Transaksi ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Biarkan Jenis Transaksi tidak dipilih
+3. Lengkapi field lain
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Jenis Transaksi: kosong</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error pada field Jenis Transaksi; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error pada field Jenis Transaksi; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-002</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Menyimpan transaksi tanpa memilih Komoditas ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Biarkan Komoditas tetap 'Pilih komoditas'
+3. Lengkapi field lain
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Komoditas: kosong</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error pada field Komoditas; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error pada field Komoditas; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-003</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Menyimpan transaksi dengan Jumlah (kg) bernilai 0 ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Isi Jumlah (kg) dengan 0
+3. Lengkapi field lain
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah (kg): 0</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error bahwa jumlah harus lebih dari 0; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error bahwa jumlah harus lebih dari 0; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="52" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-004</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Menyimpan transaksi dengan Jumlah (kg) bernilai negatif ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Isi Jumlah (kg) dengan nilai negatif
+3. Lengkapi field lain
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah (kg): -50</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error; nilai negatif tidak diterima pada field Jumlah (kg)</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error; nilai negatif tidak diterima pada field Jumlah (kg)</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="91" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-005</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Mencatat transaksi 'Keluar' dengan jumlah melebihi saldo stok saat ini menampilkan peringatan</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Pilih Jenis 'Keluar' dan Komoditas tertentu
+3. Isi Jumlah (kg) lebih besar dari saldo stok saat ini
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Beras saat ini: 100 kg | Jumlah Keluar diinput: 5.000 kg</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan peringatan terkait saldo stok tidak cukup sebelum transaksi disimpan, sesuai keterangan 'Perhatikan saldo stok saat ini sebelum mencatat transaksi keluar.'</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan peringatan terkait saldo stok tidak cukup sebelum transaksi disimpan, sesuai keterangan 'Perhatikan saldo stok saat ini sebelum mencatat transaksi keluar.'</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="65" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-006</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Menyimpan transaksi 'Keluar' tanpa memilih Tujuan Distribusi ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Pilih Jenis 'Keluar'
+3. Biarkan Tujuan Distribusi tetap 'Pilih tujuan'
+4. Lengkapi field lain
+5. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Jenis: Keluar | Tujuan Distribusi: kosong</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error pada field Tujuan Distribusi; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error pada field Tujuan Distribusi; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="52" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-007</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Menyimpan transaksi tanpa mengisi Sumber/Keterangan ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Biarkan field Sumber/Keterangan kosong
+3. Lengkapi field lain
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Sumber/Keterangan: kosong</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error pada field Sumber/Keterangan; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error pada field Sumber/Keterangan; data tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="65" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-008</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Mengunggah Foto Bukti Pengiriman dengan ukuran file lebih dari 2MB ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Lengkapi field wajib
+3. Klik 'Pilih File' pada Foto Bukti Pengiriman dan pilih file berukuran &gt; 2MB
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>File: bukti_besar.png (5 MB)</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan error bahwa ukuran file melebihi batas maksimum 2MB; file tidak terunggah dan transaksi tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan error bahwa ukuran file melebihi batas maksimum 2MB; file tidak terunggah dan transaksi tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="65" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-009</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Mengunggah Foto Bukti Pengiriman dengan format file yang tidak didukung ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Lengkapi field wajib
+3. Klik 'Pilih File' pada Foto Bukti Pengiriman dan pilih file dengan format selain jpg/png/webp
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>File: bukti.pdf</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menolak file dengan format tidak didukung dan menampilkan pesan error format file; hanya jpg, png, dan webp yang dapat diunggah</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menolak file dengan format tidak didukung dan menampilkan pesan error format file; hanya jpg, png, dan webp yang dapat diunggah</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-FN-001</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – Negatif</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Menambahkan Tujuan Distribusi dengan nama kosong ditolak sistem</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Manajemen Tujuan Distribusi
+2. Klik '+ Tambah Tujuan'
+3. Biarkan nama tujuan kosong
+4. Klik Simpan</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Nama Tujuan: kosong</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error; data tujuan tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan validasi error; data tujuan tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="52" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-FN-002</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – Negatif</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Menambahkan Tujuan Distribusi dengan nama yang sudah ada (duplikat) ditolak atau diberi peringatan</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Manajemen Tujuan Distribusi
+2. Klik '+ Tambah Tujuan'
+3. Isi nama tujuan yang sudah terdaftar
+4. Klik Simpan</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Nama Tujuan: 'Toko Barokah' (sudah ada di daftar)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan error/peringatan bahwa nama tujuan sudah terdaftar; data duplikat tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan error/peringatan bahwa nama tujuan sudah terdaftar; data duplikat tidak tersimpan</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="78" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-FN-003</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – Negatif</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Menghapus Tujuan Distribusi yang masih direferensikan oleh transaksi yang sudah tercatat tidak merusak data riwayat</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Manajemen Tujuan Distribusi
+2. Hapus tujuan yang sudah pernah dipakai pada transaksi sebelumnya
+3. Buka kembali halaman Stok Gudang dan periksa transaksi lama yang menggunakan tujuan tersebut</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan yang dihapus: 'MBG Dapur 2' (sudah pernah dipakai)</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Riwayat transaksi lama tetap menampilkan nama tujuan 'MBG Dapur 2' tanpa error, meskipun tujuan tersebut sudah dihapus dari daftar dan tidak lagi muncul di dropdown untuk transaksi baru</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Riwayat transaksi lama tetap menampilkan nama tujuan 'MBG Dapur 2' tanpa error, meskipun tujuan tersebut sudah dihapus dari daftar dan tidak lagi muncul di dropdown untuk transaksi baru</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="65" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-FN-010</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Negatif</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Detail transaksi 'Keluar' tanpa foto form menampilkan pesan yang sesuai</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik ikon mata pada transaksi berjenis 'Keluar' yang TIDAK memiliki foto form
+2. Amati bagian Foto Bukti pada halaman detail</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi: Keluar, Gabah, 100 kg, tanpa foto form</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan informatif seperti 'Foto bukti tidak tersedia'; tidak menampilkan ikon gambar rusak (broken image) atau error tampilan</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menampilkan pesan informatif seperti 'Foto bukti tidak tersedia'; tidak menampilkan ikon gambar rusak (broken image) atau error tampilan</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -2356,8 +4522,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -2377,7 +4543,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>SIMHPSB Web</t>
+          <t>SIMHP Web</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2413,7 +4579,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Description</t>
@@ -2435,7 +4601,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Test Objective</t>
@@ -2457,6 +4623,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
@@ -2499,7 +4666,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="78" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>TC-AS-EC-001</t>
@@ -2532,18 +4699,18 @@
           <t>Panel Ringkasan menampilkan 0 untuk semua kategori; tabel riwayat menampilkan pesan 'Belum ada data alert' atau tabel kosong; tidak ada error atau crash</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Halaman Alert Stok dibuka di environment tanpa data alert. Panel Ringkasan menampilkan angka 0 untuk semua kategori dan tabel riwayat menampilkan area kosong. Halaman tidak crash.</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Panel Ringkasan menampilkan 0 untuk semua kategori; tabel riwayat menampilkan pesan 'Belum ada data alert' atau tabel kosong; tidak ada error atau crash</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TC-AS-EC-002</t>
@@ -2576,18 +4743,18 @@
           <t>Alert TIDAK terpicu karena stok tidak di bawah batas minimum; status tetap normal; tidak ada baris baru di riwayat alert</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Stok Beras diatur tepat 500 kg dan batas minimum juga 500 kg. Tidak ada alert baru yang muncul di riwayat dan kartu Beras tidak berubah ke status 'Kritis' karena stok tidak di bawah batas.</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Alert TIDAK terpicu karena stok tidak di bawah batas minimum; status tetap normal; tidak ada baris baru di riwayat alert</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="65" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TC-AS-EC-003</t>
@@ -2620,18 +4787,18 @@
           <t>Alert baru dengan status 'Aktif' muncul di riwayat; badge counter 'Alert Stok' di sidebar bertambah; panel Ringkasan menambah 1 di 'Alert Aktif'</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Stok Beras diatur menjadi 499 kg (1 kg di bawah batas minimum 500 kg). Alert baru dengan status 'Aktif' langsung muncul di tabel riwayat dan badge angka di sidebar Alert Stok bertambah 1.</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Alert baru dengan status 'Aktif' muncul di riwayat; badge counter 'Alert Stok' di sidebar bertambah; panel Ringkasan menambah 1 di 'Alert Aktif'</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TC-AS-EC-004</t>
@@ -2664,18 +4831,18 @@
           <t>Sistem menyimpan tanpa error; konfirmasi simpan berhasil ditampilkan; tidak ada alert duplikat atau perubahan aneh</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>Batas minimum Beras diubah dari 500 kg ke 500 kg (nilai sama). Sistem menerima dan menyimpan tanpa error, muncul konfirmasi sukses. Tidak ada perubahan kondisi alert.</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Sistem menyimpan tanpa error; konfirmasi simpan berhasil ditampilkan; tidak ada alert duplikat atau perubahan aneh</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>TC-AS-EC-005</t>
@@ -2709,18 +4876,18 @@
           <t>Halaman load dengan waktu wajar (&lt; 5 detik); scroll tabel lancar; filter berfungsi normal; tidak ada timeout atau freeze</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Riwayat alert dengan 50+ entri dibuka. Halaman load dalam waktu normal, scroll tabel berjalan lancar, dan filter dropdown tetap berfungsi. Tidak ada freeze atau timeout.</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Halaman load dengan waktu wajar (&lt; 5 detik); scroll tabel lancar; filter berfungsi normal; tidak ada timeout atau freeze</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>TC-AS-EC-006</t>
@@ -2752,12 +4919,500 @@
           <t>Badge merah di ikon Alert Stok sidebar menampilkan angka yang sama dengan jumlah Alert Aktif di panel Ringkasan Status Alert</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Badge angka merah di ikon Alert Stok sidebar menampilkan angka 3, sama persis dengan jumlah 'Alert Aktif' di panel Ringkasan Status Alert. Keduanya sinkron.</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Badge merah di ikon Alert Stok sidebar menampilkan angka yang sama dengan jumlah Alert Aktif di panel Ringkasan Status Alert</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="91" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-001</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Halaman Stok Gudang tetap stabil saat belum ada satu pun transaksi tercatat</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>1. Akses environment baru tanpa data transaksi
+2. Buka halaman Stok Gudang
+3. Amati tampilan kartu ringkasan dan tabel riwayat</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Riwayat transaksi: kosong (0 data)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Kartu ringkasan menampilkan 0 kg untuk setiap komoditas; tabel riwayat menampilkan pesan 'Belum ada data transaksi' atau tabel kosong dengan pesan informatif; tidak ada error atau crash</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Kartu ringkasan menampilkan 0 kg untuk setiap komoditas; tabel riwayat menampilkan pesan 'Belum ada data transaksi' atau tabel kosong dengan pesan informatif; tidak ada error atau crash</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-002</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi 'Keluar' yang membuat saldo stok menjadi tepat 0 kg tersimpan tanpa error</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Pilih Jenis 'Keluar' dengan Jumlah sama dengan saldo stok saat ini
+3. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Beras saat ini: 200 kg | Jumlah Keluar: 200 kg</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi tersimpan tanpa error; kolom Saldo Setelah menampilkan '0 kg'</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi tersimpan tanpa error; kolom Saldo Setelah menampilkan '0 kg'</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="91" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-003</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Saldo stok dapat bernilai negatif setelah transaksi keluar yang sangat besar, konsisten dengan modul Alert Stok</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Pilih Jenis 'Keluar' dengan Jumlah jauh melebihi saldo stok saat ini
+3. Lanjutkan penyimpanan meski telah diperingatkan
+4. Amati kolom Saldo Setelah</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Beras saat ini: 100 kg | Jumlah Keluar: 1.108.900 kg (sesuai data uji modul Alert Stok)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi tetap tersimpan; kolom Saldo Setelah menampilkan nilai negatif (mis. -1.108.800 kg) dengan format warna merah sebagai indikator kritis, sejalan dengan perilaku pada modul Alert Stok</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi tetap tersimpan; kolom Saldo Setelah menampilkan nilai negatif (mis. -1.108.800 kg) dengan format warna merah sebagai indikator kritis, sejalan dengan perilaku pada modul Alert Stok</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="65" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-004</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Riwayat transaksi dalam jumlah sangat banyak (50+ baris) halaman tetap responsif</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>1. Pastikan riwayat transaksi memiliki 50+ entri
+2. Buka halaman Stok Gudang
+3. Scroll tabel ke bawah
+4. Coba gunakan filter dan pencarian</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah riwayat transaksi: 50+ entri</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Halaman load dengan waktu wajar (&lt; 5 detik); scroll tabel lancar; filter dan pencarian tetap berfungsi normal; tidak ada timeout atau freeze</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Halaman load dengan waktu wajar (&lt; 5 detik); scroll tabel lancar; filter dan pencarian tetap berfungsi normal; tidak ada timeout atau freeze</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="65" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-005</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Membatalkan lalu langsung memulihkan transaksi yang sama secara berurutan tidak menyebabkan duplikasi atau error</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik ikon Hapus pada transaksi Aktif
+2. Segera klik ikon Restore pada baris yang sama
+3. Periksa status akhir dan Saldo Setelah</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi: status awal Aktif, dibatalkan lalu langsung dipulihkan</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Status akhir kembali menjadi 'Aktif' dengan Saldo Setelah yang konsisten dengan kondisi sebelum dibatalkan; tidak ada baris duplikat atau error tampilan</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Status akhir kembali menjadi 'Aktif' dengan Saldo Setelah yang konsisten dengan kondisi sebelum dibatalkan; tidak ada baris duplikat atau error tampilan</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-006</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Menyimpan transaksi tanpa mengisi Catatan Tambahan (field opsional) tetap berhasil tersimpan</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Lengkapi seluruh field wajib
+3. Biarkan Catatan Tambahan kosong
+4. Klik 'Simpan'</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Catatan Tambahan: kosong</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Transaksi berhasil tersimpan tanpa pesan validasi error; kolom CATATAN pada tabel riwayat menampilkan tanda '-'</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Transaksi berhasil tersimpan tanpa pesan validasi error; kolom CATATAN pada tabel riwayat menampilkan tanda '-'</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="65" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-007</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Klik tombol 'Simpan' dua kali berturut-turut secara cepat tidak menyebabkan transaksi tersimpan ganda</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik '+ Catat Transaksi'
+2. Lengkapi seluruh field wajib
+3. Klik 'Simpan' lalu segera klik lagi sebelum modal tertutup
+4. Periksa tabel riwayat transaksi</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Aksi: double-click cepat pada tombol Simpan</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Hanya satu transaksi baru yang tersimpan di tabel riwayat; tidak ada entri duplikat; Saldo Setelah berkurang/bertambah sesuai satu transaksi saja</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Hanya satu transaksi baru yang tersimpan di tabel riwayat; tidak ada entri duplikat; Saldo Setelah berkurang/bertambah sesuai satu transaksi saja</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="91" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-EC-001</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – Edge Case</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Menghapus seluruh Tujuan Distribusi yang ada (daftar kosong) tidak menyebabkan error pada form Catat Transaksi</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>1. Hapus seluruh data pada Daftar Tujuan Distribusi (jika memungkinkan di environment test)
+2. Buka halaman Stok Gudang
+3. Klik '+ Catat Transaksi' dan buka dropdown Tujuan Distribusi</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Daftar Tujuan Distribusi: kosong</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Tabel Daftar Tujuan Distribusi menampilkan pesan 'Tidak ada data' tanpa error; dropdown Tujuan Distribusi pada form Catat Transaksi menampilkan kondisi kosong/pesan informatif tanpa crash</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Tabel Daftar Tujuan Distribusi menampilkan pesan 'Tidak ada data' tanpa error; dropdown Tujuan Distribusi pada form Catat Transaksi menampilkan kondisi kosong/pesan informatif tanpa crash</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="78" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TC-TD-EC-002</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Tujuan Distribusi – Edge Case</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Menambahkan Tujuan Distribusi dengan nama yang sangat panjang tetap tampil dengan baik di tabel dan dropdown</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>1. Buka halaman Manajemen Tujuan Distribusi
+2. Klik '+ Tambah Tujuan'
+3. Isi nama tujuan dengan teks yang sangat panjang
+4. Simpan dan periksa tampilan di tabel serta dropdown Tujuan Distribusi</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Nama Tujuan: 'Gudang Penyimpanan Sementara Kecamatan Banjar Wilayah Selatan' (lebih dari 50 karakter)</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Nama tujuan tersimpan dan tampil utuh di tabel Daftar Tujuan Distribusi maupun dropdown Tujuan Distribusi tanpa terpotong atau merusak tata letak (layout) halaman</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Nama tujuan tersimpan dan tampil utuh di tabel Daftar Tujuan Distribusi maupun dropdown Tujuan Distribusi tanpa terpotong atau merusak tata letak (layout) halaman</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="78" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-008</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Status Dibatalkan pada beberapa transaksi (lebih dari satu baris) tetap konsisten setelah halaman di-reload</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>1. Batalkan 3 baris transaksi menggunakan ikon Hapus
+2. Refresh/reload halaman Stok Gudang
+3. Periksa status ketiga transaksi tersebut</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>3 transaksi dibatalkan sebelum reload</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Ketiga transaksi tetap berstatus 'Dibatalkan' dengan format tercoret setelah reload; tidak ada transaksi yang hilang, berubah status secara tidak semestinya, atau duplikat</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Ketiga transaksi tetap berstatus 'Dibatalkan' dengan format tercoret setelah reload; tidak ada transaksi yang hilang, berubah status secara tidak semestinya, atau duplikat</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="65" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>TC-SG-EC-009</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Stok Gudang – Edge Case</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Membatalkan seluruh transaksi yang tampil pada tabel tetap menampilkan seluruh baris dengan status Dibatalkan tanpa error</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>1. Klik ikon Hapus pada seluruh baris yang tampil di tabel
+2. Amati tampilan tabel setelah seluruh baris dibatalkan</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Seluruh baris pada tabel (mis. 5 dari 5 baris) dibatalkan</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Seluruh baris tetap tampil pada tabel dengan status 'Dibatalkan' dan format tercoret; tidak ada baris yang hilang, error, atau crash pada halaman</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Seluruh baris tetap tampil pada tabel dengan status 'Dibatalkan' dan format tercoret; tidak ada baris yang hilang, error, atau crash pada halaman</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>

</xml_diff>